<commit_message>
Update recommended replies in the leads-with-links file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015dXgfxu1ugCxsD9bCGxkqs
</commit_message>
<xml_diff>
--- a/lynkk-reddit-leads/results/2026-10-11/leads_with_links_2026-10-11.xlsx
+++ b/lynkk-reddit-leads/results/2026-10-11/leads_with_links_2026-10-11.xlsx
@@ -53,10 +53,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,22 +427,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="60" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,6 +509,11 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>recommended_reply_no_brand</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
@@ -551,22 +562,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Has a weekly mix of online and in-person meetings and doesn't want to leave a phone on the table, so is looking at both an online note taker and a separate recorder.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Directly asks which AI meeting note taker to use for online and in-person meetings.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Before buying a recorder, check whether your in-person meetings happen where a laptop is already open. If they do, a laptop mic recording in the browser is usually good enough for a small room, and it keeps everything in one place with your online calls, which matters more than people expect when you're searching for a follow-up two weeks later. A dedicated recorder makes sense if you meet in places with no laptop, like site visits or coffee meetings. For the online side, try one tool that records from your computer without a bot joining, and judge it on whether the summary separates decisions from action items.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Depends on where your in-person meetings happen. If there's usually a laptop on the table, try recording from that before buying a Plaud or Pocket; a laptop mic is fine for a small room, and you get everything in one app instead of two. A recorder makes more sense for cafes or site visits.
+If you want one tool for both, Lynkk is worth a look: it records Zoom, Meet and Teams calls without a bot joining, and in-person meetings straight from the browser, so it all ends up searchable in one place.</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Before buying a recorder, check whether your in-person meetings happen where a laptop is already open. If they do, a laptop mic recording is usually fine for a small room, and it keeps everything in one place with your online calls, which matters when you're hunting for a follow-up two weeks later. A dedicated recorder makes sense for site visits or coffee meetings with no laptop. For online calls, pick something that records from your computer without a bot joining, and judge it on whether the summary separates decisions from action items.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>2026-09-25T16:56:39+00:00</t>
         </is>
@@ -598,7 +615,7 @@
           <t>Party_History2839</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
@@ -616,22 +633,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Loses important details from client consultations because weeks pass between the meeting and drafting, and handwritten notes miss context.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Detailed, active evaluation with explicit questions; answer the practical questions first and avoid any compliance claims Lynkk can't back.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>On the in-person side, a laptop's built-in mic is usually fine for two or three people across a desk, but a cheap USB boundary mic in the middle of the table makes a bigger difference to transcript accuracy than switching apps. For your weeks-later problem, judge tools on what the summary keeps: decisions, open questions and action items, with timestamps that jump back to the recording so you can check the exact wording before drafting. For a fair test, run the same real consultation through two or three tools and compare them side by side. On confidentiality, ask each vendor in writing whether they train on your recordings, where data is stored and how deletion works, and get client consent on the record at the start.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>The weeks-later gap is the real test, and demos never show it. Record a consult, leave it for two weeks, then try to draft from the notes alone and see what's missing. A cheap boundary mic on the table also matters more than the app for in-person.
+For a software-only comparison against Plaud Desktop, Lynkk is one to try: it records in-person consults in the browser and video calls through a Mac app, and every point in the notes links back to the exact spot in the recording, which helps when you're drafting weeks later.</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>On the in-person side, a laptop's built-in mic is usually fine for two or three people across a desk, but a cheap USB boundary mic in the middle of the table makes a bigger difference to accuracy than switching apps. For the weeks-later problem, judge tools on what the summary keeps: decisions, open questions and action items, with timestamps that jump back to the recording so you can check exact wording before drafting. Run the same real consultation through two or three tools side by side. On confidentiality, ask each vendor in writing whether they train on recordings and how deletion works, and get client consent on the record.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>2026-10-09T18:46:17+00:00</t>
         </is>
@@ -663,7 +686,7 @@
           <t>jordanconnelly</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Any AI tool that can handle both online and offline meeting notes?</t>
         </is>
@@ -681,22 +704,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Meeting notes are scattered across Zoom, Otter and iPhone recordings, so finding something from two weeks ago means guessing which app it is in.</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Directly asks for one tool for online and in-person meetings; be honest that phone calls on an iPhone are the hard part.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>The search problem is the real cost here, so pick the tool by where everything ends up rather than by how it records. If one app holds all your notes, searching by person or project across every meeting is what saves you the digging. Online meetings and in-person ones are easy to put in one place now: record calls from your laptop without a bot and record in-person meetings from the browser or a laptop mic. Regular phone calls are the awkward part, since most meeting tools don't record a native iPhone call. A workaround is to take important calls through a laptop app like FaceTime or WhatsApp desktop so they get captured with everything else.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Phone calls are the hard part. Almost nothing can record a regular iPhone call, so the usual workaround is taking important calls on the laptop through FaceTime or WhatsApp desktop.
+For Zoom plus in-person in one place, Lynkk covers both: the Mac app picks up Zoom, Meet, Teams, FaceTime and WhatsApp calls without a bot, and in-person meetings can be recorded from the browser, all searchable together. No phone app though, so native iPhone calls stay the gap.</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Pick the tool by where everything ends up, not how it records. If one app holds all your notes, searching by person or project across every meeting is what stops the digging. Online and in-person meetings are easy to put in one place now: record calls from your laptop without a bot and in-person meetings from a laptop mic. Native iPhone calls are the hard part, since most meeting tools can't record them. A workaround is to take important calls through a laptop app like FaceTime or WhatsApp desktop so they get captured with everything else.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>2026-10-07T14:36:08+00:00</t>
         </is>
@@ -728,7 +757,7 @@
           <t>JanFromEarth</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Looking for a system-wide dictation app for Mac — no monthly subscription</t>
         </is>
@@ -746,23 +775,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Wants to type less with system-wide dictation on a Mac and doesn't want another monthly subscription.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Direct ask for Mac dictation; Lynkk's free Instant dictation fits the no-subscription wish.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Start with the built-in one: macOS Dictation works system-wide and costs nothing, so try it for a week and see where it annoys you (usually punctuation and names). If it's good enough, you're done.
 If you want something that cleans up better, Lynkk's Mac app has a free dictation mode: hold a key (fn by default), talk, and the text lands wherever your cursor is, in any app. The free Instant mode runs on the Mac and is English only; the cleaner modes that remove ums are on the paid plan, so try the free one first.</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Start with the built-in one: macOS Dictation works system-wide and costs nothing, so try it for a week and see where it annoys you (usually punctuation and names). If it's good enough, you're done.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>2026-09-06T22:52:33+00:00</t>
         </is>
@@ -794,7 +828,7 @@
           <t>FinishTough23</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Can any AI notetaker show how a decision changed across multiple meetings?</t>
         </is>
@@ -812,22 +846,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>When a decision changes across several meetings, they open summaries in date order to work out which version is current.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Asks directly whether any notetaker handles decisions across multiple meetings; be careful not to claim a dedicated decision timeline view.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>I haven't seen a tool that builds a clean decision changelog on its own, so the practical answer is a combination. First, use a notetaker whose summaries keep decisions separate from concerns and open questions, so a supplier worry never reads like a date change. Second, ask your questions across all the project's meetings rather than one, and only trust answers that cite the specific meeting and moment, so you can click through and confirm a suggestion really became an agreement. Third, when a decision changes, say it explicitly on the call, something like 'we're replacing the October launch with November because of lead times'. That one sentence makes every tool's history far more reliable.</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Summaries are bad at this because each one only knows its own meeting. What works better is asking across the whole project ('what's the current launch date and when did it change?') and only trusting answers that point to the specific meeting and moment, so you can check whether it was a real decision or just someone floating an idea.
+Lynkk's chat works roughly that way: it answers only from your own notes, finds them by project, and every answer has citations that open the note at the exact moment. Not a dedicated decision timeline, but it handles the 'what's current and why' question.</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>I haven't seen a tool that builds a clean decision changelog on its own, so the practical answer is a combination. Use a notetaker whose summaries keep decisions separate from concerns and open questions, so a supplier worry never reads like a date change. Ask questions across all of the project's meetings rather than one, and only trust answers that cite the specific meeting and moment. And when a decision changes, say it explicitly on the call: 'we're replacing the October launch with November because of lead times'. That one sentence makes every tool's history far more reliable.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>2026-09-21T06:35:54+00:00</t>
         </is>
@@ -877,7 +917,7 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Handwritten notes are too slow with several people talking, and built-in meeting transcription mixes up speaker names.</t>
         </is>
@@ -887,13 +927,18 @@
           <t>Asks directly which AI note taker to use; good fit.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>Speaker mix-ups are the main thing to test, so try each tool on a real meeting where people talk over each other, not a tidy demo. Also check whether you can jump from a line in the summary to that moment in the recording; it makes fixing a misheard word or a wrong name quick. If most of your meetings are online, a tool that records from your computer is easier than a separate recorder.
 Lynkk is one worth adding to the test: it records Zoom, Meet and Teams without a bot, keeps your own side on its own channel so it's labelled separately, and every takeaway in the summary links back to the recording.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Speaker mix-ups are the main thing to test, so try each tool on a real meeting where people talk over each other, not a tidy demo. Also check whether you can jump from a line in the summary to that moment in the recording; it makes fixing a misheard word or a wrong name quick. If most of your meetings are online, a tool that records from your computer is easier than a separate recorder.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>2026-09-11T05:36:08+00:00</t>
         </is>
@@ -925,7 +970,7 @@
           <t>BakerInfamous6110</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Do we need another AI meeting note taker for microsoft teams if we have Copilot?</t>
         </is>
@@ -943,22 +988,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Copilot only covers Teams meetings, but more customer calls now happen on links they don't own, and those are the calls they need later.</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Clear gap with built-in tools; a reply can lay out how to make the budget case.</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>If the calls you need are on customers' links, Copilot won't get you there, because it works inside meetings your tenant hosts. For the finance conversation, count how many important customer calls last month happened outside Teams, since that number is the case. The cheapest fix is usually a tool that records from the laptop itself rather than joining the meeting, so it doesn't matter whose link it is or which platform the customer picked. Keep Copilot for internal Teams meetings and only add seats for the people who take external calls, which keeps the second product small.</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Copilot only really covers meetings your tenant hosts, so customer calls on their Zoom links fall through. For the budget conversation, count how many important customer calls last month were outside Teams; that number usually settles it.
+If you add something, pick a tool that records from the laptop instead of joining as a bot, so it doesn't matter whose link it is. Lynkk's Mac app works like that across Zoom, Meet, Teams and Webex (Apple silicon Macs only).</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>If the calls you need are on customers' links, Copilot won't get you there, because it works inside meetings your tenant hosts. For the finance conversation, count how many important customer calls last month happened outside Teams; that number is the case. The cheapest fix is usually a tool that records from the laptop itself rather than joining the meeting, so it doesn't matter whose link it is. Keep Copilot for internal Teams meetings and only add seats for the people who take external calls.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>2026-10-07T06:10:07+00:00</t>
         </is>
@@ -1008,23 +1059,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Hit Wispr Flow's free weekly dictation limit and wants something free or cheap on the Mac.</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>Direct ask for Mac dictation; Lynkk's free Instant mode fits. Don't promise unlimited.</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>Worth knowing what you liked about Wispr: if it's the cleanup (removing ums, fixing punctuation), the free options mostly don't do that well; if it's just speed and working in every app, plenty of free ones are fine.
 Lynkk's Mac app is one to try: hold a key (fn by default), talk, and the text appears wherever your cursor is. The basic Instant mode is free and runs on the Mac (English only), while the cleanup modes that remove ums are on the paid plan.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Worth knowing what you liked about Wispr: if it's the cleanup (removing ums, fixing punctuation), the free options mostly don't do that well; if it's just speed and working in every app, plenty of free ones are fine.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>2026-08-11T13:58:56+00:00</t>
         </is>
@@ -1074,23 +1130,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Two clients want Zoom notes with central retention and control over who records, and they don't want to support two products.</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>Clear buyer asking about admin control; note the 10 seat cap honestly.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>What usually breaks by month three is the stuff users can change without the admin: personal accounts recording customer calls, notes shared by public link, and local files left on laptops. Check three things on any tool: whether the company can see and retain notes made on company accounts, whether sharing links can be revoked, and whether audio lands in the cloud workspace rather than Downloads.
 For small teams, Lynkk's workspaces handle that split well: admins can read workspace-visible notes, every admin read is logged, and people can mark a note personal. They cap at 10 seats though, so only if each client team is small.</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>What usually breaks by month three is the stuff users can change without the admin: personal accounts recording customer calls, notes shared by public link, and local files left on laptops. Check three things on any tool: whether the company can see and retain notes made on company accounts, whether sharing links can be revoked, and whether audio lands in the cloud workspace rather than Downloads.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>2026-10-06T15:39:36+00:00</t>
         </is>
@@ -1140,22 +1201,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Takes lots of notes on in-person sales calls because they are forgetful, then spends a lot of time entering them into Salesforce and writing follow-up emails.</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Clear ask for tools; be honest that CRM entry would still be manual with Lynkk.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Since your customers are fine with recording, I'd skip handwriting conversion and record the meeting instead. Handwriting to text still leaves you summarizing your own scribbles, while a recording gives you a full transcript and a summary with next steps you didn't have to write. Ask any tool you try to separate decisions, action items with owners, and open questions, because that structure maps straight onto a follow-up email. For Salesforce, check whether the tool actually syncs fields or just exports text, since many only do the second. Spend five minutes right after each meeting confirming next steps while it's fresh, and the CRM update gets much faster.</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>If customers are fine with recording, skip the tablet and handwriting route; you'd still be summarizing your own notes afterwards. Record the meeting, let the tool pull out next steps, and the follow-up email is mostly written.
+For in-person meetings from a laptop, Lynkk records in the browser and gives you decisions and action items with owners and due dates. It doesn't sync to Salesforce, so check that part with any tool you try, since most only hand you text.</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Since your customers are fine with recording, I'd skip handwriting conversion and record the meeting instead. Handwriting to text still leaves you summarizing your own scribbles, while a recording gives you a transcript and a summary with next steps you didn't write. Ask any tool to separate decisions, action items with owners and open questions, because that maps straight onto a follow-up email. For Salesforce, check whether a tool actually syncs fields or just exports text. Spend five minutes right after each meeting confirming next steps while it's fresh.</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>2026-09-19T00:58:59+00:00</t>
         </is>
@@ -1187,7 +1254,7 @@
           <t>jnjsch</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Best workflow for recording in-person/online meetings and syncing transcripts + AI notes into Obsidian? (Granola alternative)</t>
         </is>
@@ -1205,23 +1272,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Their Granola plus Obsidian sync setup broke after Granola locked down API access, so they need a new way to capture meetings into their vault.</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Asks directly for a Granola alternative; be honest that the Obsidian sync part needs checking.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>Since the sync part is what broke, I'd pick capture and Obsidian export separately. For capture, anything that records your mic and system audio without a bot covers online calls, and a laptop mic is fine for in-person. For the vault, the most durable setup is a tool that gives you plain text or Markdown you can paste or drop into a folder, so a plugin breaking can't strand your notes again.
 Lynkk is one to look at for the capture side: no-bot recording for calls, in-person from the browser, and summaries with decisions and action items. Check how you'd get notes into the vault before committing, since there's no Obsidian plugin.</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Since the sync part is what broke, I'd pick capture and Obsidian export separately. For capture, anything that records your mic and system audio without a bot covers online calls, and a laptop mic is fine for in-person. For the vault, the most durable setup is a tool that gives you plain text or Markdown you can paste or drop into a folder, so a plugin breaking can't strand your notes again.</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>2026-08-15T22:28:33+00:00</t>
         </is>
@@ -1271,22 +1343,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>Tired of going back through long meetings to find small details.</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>Asks what AI note apps people use for meetings, though the sub is about a hardware recorder so tone should stay helpful rather than salesy.</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>For finding small details later, the thing that matters most is whether the summary links back to the exact moment in the recording. Takeaways with timestamps you can click save a lot of scrubbing, and so does being able to search across all your meetings instead of one at a time. For long meetings, test with a real 60 to 90 minute call rather than a short demo, since that is where summaries tend to get vague. Also check how each tool labels speakers, because a decision attributed to the wrong person is worse than no note at all.</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>The biggest difference on long meetings is whether you can jump from a line in the summary straight to that moment in the audio; it saves a lot of scrubbing. Test with a real 90-minute meeting, not a short demo, because that's where summaries go vague.
+Lynkk does the timestamp-to-audio part well: every takeaway plays the recording from that moment. It's Mac, Chrome and web rather than a pocket recorder, so it's a different setup from Plaud.</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>For finding small details later, the thing that matters most is whether the summary links back to the exact moment in the recording. Takeaways with clickable timestamps save a lot of scrubbing, and so does searching across all your meetings at once. For long meetings, test with a real 60 to 90 minute call rather than a short demo, since that is where summaries get vague. Also check how each tool labels speakers, because a decision attributed to the wrong person is worse than no note at all.</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>2026-10-08T20:54:19+00:00</t>
         </is>
@@ -1318,7 +1396,7 @@
           <t>Then_Date1452</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>One AI meeting note taker for Microsoft Teams and all the zoom links?</t>
         </is>
@@ -1336,22 +1414,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>Teams' built-in notes miss the roughly 40 percent of customer calls that happen on Zoom, and adding a second tool means two archives, trainings and retention policies.</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Clear cross-platform need; a reply can cover what to test before rolling out one tool, and should note the 10 seat workspace limit if Lynkk is named.</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>One tool for both is doable, but test it on the external calls first, since those are what the built-in option misses. Three things tend to break in practice: customers' Zoom settings blocking or delaying bots in the waiting room, so check whether the tool can also record from the user's own machine; recordings landing in different places depending on who hosted the call; and retention settings that differ between personal and company accounts. Run a two-week pilot with the people who take the most Zoom calls and count how many external calls actually got captured. That number will tell you more than any feature list, and it is the one users complain about when they switch back.</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>What usually breaks is external Zoom calls where the host's settings hold bots in the waiting room, so make sure whatever you pick can also record from the user's own machine. Then pilot it for two weeks with the heaviest Zoom users and count how many external calls actually got captured.
+Lynkk handles both cases in one archive: a bot for Teams, Zoom and Meet, plus a no-bot Mac app and Chrome extension for when bots get blocked. Workspaces cap at 10 seats, so it only fits a small team.</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>One tool for both is doable, but test it on the external calls first, since those are what the built-in option misses. Three things tend to break: customers' Zoom settings blocking or delaying bots in the waiting room, so check whether the tool can also record from the user's own machine; recordings landing in different places depending on who hosted; and retention settings that differ between personal and company accounts. Run a two-week pilot with the heaviest Zoom users and count how many external calls actually got captured.</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t>2026-09-29T16:48:48+00:00</t>
         </is>
@@ -1401,22 +1485,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>AI note takers summarize decently but they still go back through the notes to double check everything.</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>Asks which AI meeting note taker people use and whether any saves time without full manual review.</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Honestly some review is still worth doing, but it can be a two-minute skim instead of a reread. What cuts the cleanup most is a summary that keeps decisions, action items and open questions as separate lists, plus timestamps on each item that jump to the moment in the recording, so you only check the items that look off. Saying owners and deadlines out loud near the end of the call also helps a lot, since the tool picks up explicit commitments far better than vague ones. If a tool can't show you where in the call an action item came from, that's usually the one that leaves you double checking everything.</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Some review will always be needed, but it can be a two-minute skim. What cuts it down most is every action item having a timestamp you can click to hear the original moment, so you only check the ones that look off. Saying owners and dates out loud at the end of the call helps a lot too.
+Lynkk is built around that click-to-check idea: decisions, action items with owners and due dates, and open questions, each linked back to the recording.</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Some review is still worth doing, but it can be a two-minute skim instead of a reread. What cuts cleanup most is a summary that keeps decisions, action items and open questions as separate lists, with timestamps on each item that jump to the moment in the recording, so you only check what looks off. Saying owners and deadlines out loud near the end of the call also helps, since tools pick up explicit commitments far better than vague ones. If a tool can't show where an action item came from, that's usually the one that leaves you double checking everything.</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>2026-09-17T17:48:26+00:00</t>
         </is>
@@ -1448,7 +1538,7 @@
           <t>Big-Personality-9618</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Otter alternative for business when everyone has a separate account?</t>
         </is>
@@ -1466,23 +1556,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Individual Otter accounts mean retention varies, visibility is limited and offboarding means chasing accounts.</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Real business need; be honest that importing old Otter history isn't something Lynkk claims.</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>On the migration worry: plan to export each person's Otter history to files before switching and store it centrally, rather than expecting a new tool to import it. Most don't do that cleanly, and it means the old history isn't hostage to whichever tool you choose. Then switch new meetings only, so people aren't asked to change everything at once.
 For the management side on small teams, Lynkk's workspaces cover what you listed: colleagues join by company email domain, admins can read workspace-visible notes with every admin read logged, and people can still mark a note personal. They cap at 10 seats, so it fits small clients only.</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>On the migration worry: plan to export each person's Otter history to files before switching and store it centrally, rather than expecting a new tool to import it. Most don't do that cleanly, and it means the old history isn't hostage to whichever tool you choose. Then switch new meetings only, so people aren't asked to change everything at once.</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>2026-09-28T11:00:38+00:00</t>
         </is>
@@ -1532,23 +1627,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Starting a new job and worried about remembering everything from meetings and training.</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>Asks directly for recommendations; keep it warm and practical.</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>For a new job, the biggest win is being able to search everything later instead of relying on memory, so whatever you pick, make sure you can find 'what did they say about X' weeks later. Ask before recording people, and for training sessions it's usually welcome. Also, re-read the action items the same day; that's when it actually sticks.
 Lynkk is one to try: it records Zoom, Meet and Teams without a bot joining, gives you takeaways and action items after each meeting, and you can search across all of them. There's a free plan, so you can see if it suits you before paying.</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>For a new job, the biggest win is being able to search everything later instead of relying on memory, so whatever you pick, make sure you can find 'what did they say about X' weeks later. Ask before recording people, and for training sessions it's usually welcome. Also, re-read the action items the same day; that's when it actually sticks.</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>2026-09-03T13:06:59+00:00</t>
         </is>
@@ -1598,23 +1698,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Jamie is too expensive and Otter can't tell speakers apart; wants botless recording, named speakers from the calendar, an MCP connection to ChatGPT, under $10 a month.</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Clear buyer, but Lynkk only clearly meets the botless requirement; be honest about the rest.</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>Speaker naming is usually where the cheaper tools fall down, so I'd test that first with a real three-person call before anything else. Botless capture is common now, so it shouldn't be the deciding factor. And check whether the MCP access is on the plan you'd actually pay for, since a lot of tools keep it for higher tiers.
 Lynkk is another one to put in the test: it records without a bot from a Mac app or a Chrome extension and labels your own side of the call separately. Worth checking its pricing and integrations against your list directly.</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Speaker naming is usually where the cheaper tools fall down, so I'd test that first with a real three-person call before anything else. Botless capture is common now, so it shouldn't be the deciding factor. And check whether the MCP access is on the plan you'd actually pay for, since a lot of tools keep it for higher tiers.</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>2026-09-11T06:28:40+00:00</t>
         </is>
@@ -1646,7 +1751,7 @@
           <t>Sash19</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Any Fathom AI alternatives that work better with agent workflows?</t>
         </is>
@@ -1664,22 +1769,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>Getting enough context from past meetings for follow-ups, tasks and older decisions means moving transcripts around by hand.</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>Asks what people use when meeting data feeds an agent; a reply can explain the trade-off between exporting data and asking questions inside the notes tool.</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Two setups seem to work. One is piping transcripts into your agent through an integration like the MCP route you're testing, which is flexible but means your agent does the retrieval work. The other is asking questions directly in the notes tool, if it can search across all your meetings by person, company or project and cite the moment in the recording. For follow-ups and older decisions, the second is often enough and avoids moving transcripts around. Whichever you pick, make sure decisions and action items are stored as structured items rather than buried in summary prose, because that's what makes them retrievable months later.</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Depends whether you need the meeting data inside your own agent or just need answers. If it's mostly 'what did we decide with X' and 'what's still open', asking inside the notes tool is simpler than wiring transcripts into an agent. If the agent has to act on it with other context, your MCP route makes sense.
+For the first case, Lynkk lets you ask across all your notes, gives answers that link back to the moment, and can create a Jira issue from there. You can ask it from Slack too.</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Two setups seem to work. One is piping transcripts into your agent through an integration like the MCP route you're testing, which is flexible but means your agent does the retrieval. The other is asking questions directly in the notes tool, if it can search across all meetings by person, company or project and cite the moment in the recording. For follow-ups and older decisions, the second is often enough. Either way, make sure decisions and action items are stored as structured items rather than buried in summary prose.</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>2026-09-25T17:06:49+00:00</t>
         </is>
@@ -1711,7 +1822,7 @@
           <t>lebron7</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Are AI note-taking tools actually better than taking notes yourself?</t>
         </is>
@@ -1729,22 +1840,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>Doesn't fully trust AI meeting notes without checking, because small details matter more than the summary.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Asks what tool people use and raises the trust problem, which has a practical answer.</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Checking is the right instinct. What made it workable for me is a tool where every takeaway and action item carries a timestamp you can click to hear the original moment, so verifying a detail takes ten seconds instead of rereading the transcript. Also worth making a habit of saying decisions and owners out loud at the end of the call, since the summary picks those up far more reliably than something mentioned in passing. I'd still skim action items right after the meeting while it's fresh, then trust the rest as a searchable record rather than a final document.</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Checking is the right instinct. What makes it workable is clicking a line in the summary and hearing the original moment, so a detail takes seconds to verify instead of rereading the transcript. Trust the summary for the gist and the recording for names and numbers.
+Lynkk does the click-to-hear part: every takeaway and action item has a timestamp that plays the recording, and you can search across all your meetings afterwards.</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Checking is the right instinct. What made it workable for me is a tool where every takeaway and action item carries a timestamp you can click to hear the original moment, so verifying a detail takes ten seconds instead of rereading the transcript. Also make a habit of saying decisions and owners out loud at the end of the call, since summaries pick those up far more reliably than something mentioned in passing. Skim action items right after the meeting, then treat the rest as a searchable record rather than a final document.</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>2026-10-08T22:09:33+00:00</t>
         </is>
@@ -1776,7 +1893,7 @@
           <t>Morphius007</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>My AI summarized a meeting and invented an action item that committed us to a go-live date.</t>
         </is>
@@ -1794,22 +1911,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>An AI meeting summary invented an action item that committed the team to a go-live date nobody agreed to.</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>Asks a concrete question about constraining AI action items; practical advice fits well.</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>The most reliable fix is evidence, not banned words. Require every action item to link to the moment in the recording or the quote it came from, and treat any item without one as a draft. That makes an invented deadline obvious in seconds because there's nothing to click. Second, split the output into decisions, action items and open questions, and have the owner confirm their own items before anything goes on the board, rather than the PM approving everyone's. Third, end calls with a 60 second recap where someone says the owners and dates out loud. Summaries stick much closer to commitments that were stated explicitly.</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>That 'inferred urgency' is why action items need a source. Simplest rule: every action item links to the moment it was said, and anything without a source stays a draft. That catches invented deadlines in seconds. Also have owners confirm their own items instead of the PM approving everything.
+Lynkk works this way: each action item carries a timestamp back to the recording, and nothing goes to Jira unless someone sends it by hand.</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>The most reliable fix is evidence, not banned words. Require every action item to link to the moment in the recording or the quote it came from, and treat any item without one as a draft. That makes an invented deadline obvious in seconds. Second, split output into decisions, action items and open questions, and have each owner confirm their own items before anything goes on the board. Third, end calls with a 60-second recap where someone says owners and dates out loud. Summaries stick much closer to commitments that were stated explicitly.</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>2026-09-18T14:51:22+00:00</t>
         </is>
@@ -1841,7 +1964,7 @@
           <t>Party_History2839</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
@@ -1859,18 +1982,28 @@
           <t>check_rules</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>Worried they bought into the Plaud ecosystem right before a decline, and needs to make a recommendation to the firm.</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>Same person as the main lawyers post; reply to the main post instead of here.</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Fair worry. Whatever you pick, export your recordings regularly so you're never stuck, and do a short side-by-side with a second tool before recommending anything firm-wide.
+If you want a software-only option to compare, Lynkk is one: no hardware to bet on, in-person recording from the browser, and calls through a Mac app.</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Reasonable worry for a firm-wide decision. A few things that protect you whichever tool you pick: export your recordings and transcripts regularly so you're never locked in, run a two-week pilot of two tools on real consultations before committing, and make the choice on what the notes look like weeks later, not on the first demo. A tool that's useful to you today is fine as long as leaving it is cheap.</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t>2026-10-10T03:47:30+00:00</t>
         </is>
@@ -1921,13 +2054,23 @@
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>Same person as the stronger r/AIAssisted post; reply there first.</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Mostly depends on whether you have in-person meetings too. If you do, keep everything in one tool, otherwise you end up searching two places later.
+Lynkk is one that covers both: calls without a bot from a Mac app or Chrome extension, and in-person meetings from the browser.</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Depends on your mix. For online calls, something that records from your computer without a bot is the least awkward with clients. If you also have in-person meetings, keep them in the same tool so you can search everything in one place later. Whatever you try, judge it on whether the summary separates decisions from action items and links back to the recording.</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
         <is>
           <t>2026-09-28T09:05:53+00:00</t>
         </is>
@@ -1959,7 +2102,7 @@
           <t>Morphius007</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>My meeting-notes AI invented action owners who were not even in the meeting.</t>
         </is>
@@ -1977,18 +2120,28 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>AI meeting summary assigned action items to people who never joined the meeting.</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>Same person as the stronger invented deadline post; reply there first.</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Attendee-only is a good guardrail, but go one step further: only set an owner when someone actually said it, with a link to that moment, and otherwise mark it 'owner needed'. A 30-second recap at the end ('Priya has the roadmap, Friday') removes most of the guessing.
+Tools that link each action item to the recording make this quick to check; Lynkk does that for every action item.</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Attendee-only owners is a sensible rule, but the stronger check is evidence: an owner should only be set when someone said it in the meeting, with a link to that moment. Anything else becomes 'owner needed' rather than a name. Then have the named owner confirm the item themselves before it goes anywhere. A quick verbal recap at the end of the call ('Priya has the roadmap, due Friday') removes most of the guessing the model is doing.</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t>2026-09-20T14:17:01+00:00</t>
         </is>
@@ -2020,7 +2173,7 @@
           <t>Comfortable-Pay611</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>What’s the most useful thing your AI recorder gives you after a meeting?</t>
         </is>
@@ -2038,18 +2191,27 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>Still writes the follow-up email by hand after getting a transcript, summary and action items.</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>Good engagement thread; a practical answer fits better than a pitch.</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>A follow-up that's basically ready to send wins for most people, but only if it's built from the action items rather than the summary. The summary is for whoever missed the meeting; the action items with owners and dates are what you actually send to the client. Asking for 'decisions, action items with owner and date, and open questions' as the output shape gets you most of the way to that email.</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>A follow-up that's basically ready to send wins for most people, but only if it's built from the action items rather than the summary. The summary is for whoever missed the meeting; the action items with owners and dates are what you actually send to the client. Asking for 'decisions, action items with owner and date, and open questions' as the output shape gets you most of the way to that email.</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t>2026-10-11T12:28:04+00:00</t>
         </is>
@@ -2081,7 +2243,7 @@
           <t>Big-Personality-9618</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Other alternative for business when everyone has a separate account?</t>
         </is>
@@ -2105,8 +2267,13 @@
           <t>Same person as the other r/Entrepreneurs post; reply there.</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>No separate reply: Same person as the other r/Entrepreneurs post; reply there.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
         <is>
           <t>2026-09-28T06:45:31+00:00</t>
         </is>
@@ -2138,7 +2305,7 @@
           <t>Party_History2839</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
@@ -2156,18 +2323,28 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>Feels Plaud is drifting toward an enterprise agent platform and away from the recording and summarizing they bought it for.</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Same person as the main lawyers post; reply to the main post instead.</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Makes sense. If what you need is record, transcribe and summarize reliably, the agent features are noise. Write down the three things you actually rely on and test alternatives against only those.
+Lynkk is worth adding to that test since it sticks to the core: recording, transcript, and a brief that links back to the audio.</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>That's a fair reason to look around: if what you need is recording, transcription and a reliable summary, a tool that stays focused on that is worth more than agent features you won't use. Before switching, write down the three things you rely on most and test any alternative against exactly those on a real consultation.</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t>2026-10-10T04:22:35+00:00</t>
         </is>
@@ -2223,8 +2400,13 @@
           <t>Same person as the stronger r/AiNoteTaker post; reply there.</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>No separate reply: Same person as the stronger r/AiNoteTaker post; reply there.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
         <is>
           <t>2026-09-28T08:25:05+00:00</t>
         </is>
@@ -2256,7 +2438,7 @@
           <t>Overall_Fold7937</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
@@ -2274,18 +2456,28 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>Plaud transcription accuracy has dropped, especially on mixed language meetings, so they spend time correcting it.</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>Real frustration but not asking for alternatives, and it's in the Plaud sub; low priority.</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Mixed language is rough for most engines. Setting the languages explicitly, if your tool allows it, and adding names and terms to a custom vocabulary usually helps more than anything.
+For a comparison point, Lynkk transcribes 17 languages with auto-detect and has a custom words list. Worth one side-by-side on a mixed meeting.</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Mixed-language meetings are hard for most transcription engines. Two things that help: check whether the tool lets you set the languages up front instead of auto-detecting each segment, and add a custom vocabulary for names and terms that keep coming out wrong. Also compare against a short sample you transcribe by hand, so you know whether it's the audio or the model.</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t>2026-10-10T12:43:46+00:00</t>
         </is>
@@ -2317,7 +2509,7 @@
           <t>belligerent_vogue</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Is there an AI tool that can tell me exactly where a sales negotiation went wrong?</t>
         </is>
@@ -2335,18 +2527,28 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>Can't spend all day listening to hour-long sales calls to find the two minutes where a negotiation went wrong.</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>Real need, but they want conversation intelligence for coaching, which goes beyond what Lynkk claims.</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>Start smaller than a coaching platform. Take five lost deals and five won ones and only listen from the first price mention onward; patterns show up faster than you'd expect.
+To cut the listening time, a tool with timestamped takeaways helps you jump straight to the price discussion. Lynkk does that, though it isn't a coaching tool, so it helps with the review time rather than scoring reps.</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Start smaller than a full coaching platform. Pick five lost deals and five won ones, and only review the stretch from first price mention to the end of that discussion. Mark where the client's tone changed and what the rep said just before. Patterns show up fast across ten calls. Then build a short checklist from what your top reps do in that moment and score new calls against it. Whatever tool you test, judge it on whether it finds those moments for you with a timestamp you can jump to.</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t>2026-10-09T16:45:33+00:00</t>
         </is>
@@ -2396,18 +2598,28 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>Unsure an AI meeting assistant saves work after the call when someone still has to check whether a suggestion was really a decision.</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>Discussion question, not a tool request; a reply could share practical habits.</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>The summary itself rarely saves time. What helps is when 'we could try this' gets filed as an open question instead of a decision, and you can click back to hear how it was actually said.
+Lynkk splits decisions, action items and open questions that way and records without a bot, similar to what you like about Bluedot. Curious what others find actually gets opened after the meeting.</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>The useful part for most people isn't the summary, it's the structure: decisions in one list, action items with owners in another, open questions in a third. 'We could try this' should land in open questions, not decisions. If a tool keeps those apart and links each item to the moment in the recording, checking takes a minute and the summary actually gets opened. If it just produces prose, it becomes another document nobody reads.</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>2026-10-05T22:31:21+00:00</t>
         </is>
@@ -2457,18 +2669,27 @@
           <t>no</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>Construction PM on four projects doing meeting minutes and everything else alone, with a newborn on the way.</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>Engagement fit: meeting minutes is a concrete win to suggest among broader advice.</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Meeting minutes is the easiest one to take off your plate first. Record the OAC and sub meetings (with permission), let a tool draft minutes with action items, owners and dates, then spend five minutes correcting it before it goes out. That alone usually gives back a few hours a week. Copilot can help with drafting submittal logs and emails if you already have it. Congrats on the newborn, and protect that time off.</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Meeting minutes is the easiest one to take off your plate first. Record the OAC and sub meetings (with permission), let a tool draft minutes with action items, owners and dates, then spend five minutes correcting it before it goes out. That alone usually gives back a few hours a week. Copilot can help with drafting submittal logs and emails if you already have it. Congrats on the newborn, and protect that time off.</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
         <is>
           <t>2026-08-12T02:29:05+00:00</t>
         </is>

</xml_diff>